<commit_message>
feat: highlight-to-teach suffix removal, -C panel side default, plain-language rule descriptions
</commit_message>
<xml_diff>
--- a/tests/fixtures/duplicate-parents.xlsx
+++ b/tests/fixtures/duplicate-parents.xlsx
@@ -451,7 +451,7 @@
         <v/>
       </c>
       <c r="F2" s="2" t="str">
-        <v>MTR-A</v>
+        <v>MTR-1</v>
       </c>
       <c r="G2" s="2" t="str">
         <v>10</v>
@@ -474,7 +474,7 @@
         <v/>
       </c>
       <c r="F3" s="2" t="str">
-        <v>MTR-B</v>
+        <v>MTR-2</v>
       </c>
       <c r="G3" s="2" t="str">
         <v>11</v>
@@ -497,7 +497,7 @@
         <v/>
       </c>
       <c r="F4" s="2" t="str">
-        <v>MTR-C</v>
+        <v>MTR-3</v>
       </c>
       <c r="G4" s="2" t="str">
         <v>12</v>

</xml_diff>